<commit_message>
Replace markdown report with a Relatório sheet in the xlsx
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LHSta4BSCkfbiPMDEfDYZf
</commit_message>
<xml_diff>
--- a/analysis/atlas_clusters_vs_fnp.xlsx
+++ b/analysis/atlas_clusters_vs_fnp.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atlas 2025 - clusters (MRT)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FNP - regiões e municípios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparação por UF" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achados Atlas 2023" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Razão 2025 sobre 2023" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatório" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atlas 2025 - clusters (MRT)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FNP - regiões e municípios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparação por UF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achados Atlas 2023" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Razão 2025 sobre 2023" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51,8 +52,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,6 +422,263 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Seção</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Detalhe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>PDFs indisponíveis</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Os PDFs do Atlas 2023/2025 não estavam disponíveis (não anexados; gov.br bloqueado pela rede do ambiente). A conferência Excel x PDF NÃO foi feita e os municípios de cada MRT NÃO foram extraídos (o Excel do Atlas não os contém). Tudo abaixo vem apenas dos dois Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Atlas 2025</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Estrutura</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>239 MRTs, 27 UFs, 1.954 linhas, 1 linha 'Geral' por MRT: bate com o título da planilha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Atlas 2025</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>A conferir no PDF</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>18 linhas com VTN &gt; VTI (ex.: PB-1803, GO-401 Pecuária, MS-1605 Pecuária, SE-2304/2305 Geral); 3 pares (MRT, tipologia) duplicados (RS-1106 Agrícola, DF-2808/GO-2808); 38 MRTs com 'Geral' fora do intervalo das tipologias nível 1; outliers extremos (MG-606 Varginha Não Agrícola R$ 1,15 mi/ha; PI-2405 R$ 320/ha).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Atlas 2023</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>UF errada</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>9 MRTs com UF divergente do código (+1 interestadual ambíguo, 2802 Formoso): 1501 Sul Amazonense (rotulado Acre; é AM), 1205 Metropolitano (Amapá; é MA), 3001 Baixo Amazonas (Amazonas; é PA), 1905 (Ceará; é RN), 611 Timóteo (Maranhão; é MG), 701 Vale do Paraíba (Paraíba; é RJ), e 1601 Corumbá, 1607 Paranaíba, 1613 Ivinhema rotulados como Mato Grosso (são MS). 803 Mogiana está como Espírito Santo, mas o código 8xx parece SP (código inexistente em 2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Atlas 2023</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Blocos misturados</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>48 dos 51 MRTs têm 2-3 linhas 'Geral'. Só o 1º bloco casa com o MRT nomeado (razão 2025/2023 ~1,28); os demais parecem de MRTs vizinhos sem cabeçalho (ex.: 1205 Metropolitano com VTI 233 mil e 4,9 mil/ha; MT Pantanal com Agricultura a R$ 50-87 mil/ha). Consistente com o aviso da planilha (só ~50 de 184 MRTs em formato tabular). Os dados de MT 2023 estão contaminados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Atlas 2023</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>4 linhas com VTN média &gt; VTI média; 1 com VTI média fora de [mín, máx]; 3 com VTN fora; tipologias truncadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2023 -&gt; 2025</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Valores indexados</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Em 100 de 193 linhas comparáveis a razão 2025/2023 é idêntica (x1,2836: 53; x1,1200: 25; x1,3124: 22). Parece correção por índice, não preço novo de mercado. Se confirmado no PDF, não usar essa variação como sinal de mercado nesses MRTs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Clusters</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Granularidade</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Atlas 2025: 239 MRTs (inclui DF), 27 UFs. FNP: 133 regiões, 26 UFs, 5.494 municípios (sem DF). Atlas é ~1,8x mais granular, mas desigual: SC 16 x 4, GO 18 x 7, ES 13 x 3, TO 13 x 3; SP é o inverso (6 x 14); PR 8 x 9; MT 11 x 11; RR 2 x 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Clusters</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Divisas de UF</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Alguns MRTs do Atlas cruzam UFs (Unaí/Cristalina GO+MG, Mambaí/Formoso GO+MG, 'Distrito Federal' GO+DF). Regiões FNP nunca cruzam UF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Clusters</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Nomes (exemplo MT)</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Atlas-MT: Pantanal, Sudoeste, Parecis, Capital, Médio Araguaia, Sul, Norte Araguaia, Norte, Centro, Oeste, Noroeste. FNP-MT: Cáceres, Cuiabá, Rondonópolis, Alto Araguaia, Pontes e Lacerda, Tangará da Serra, Sinop, Barra do Garças, Aripuanã, Alta Floresta, Vila Rica. Lógicas aparentemente diferentes (Atlas: zonas homogêneas de valor/uso; FNP: polos/áreas de influência).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Clusters</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Conclusão provisória</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Não misturar os dois sistemas diretamente. A viabilidade de cruzar (município -&gt; MRT e -&gt; região FNP, medir sobreposição) só pode ser testada com a lista de municípios dos MRTs, que está nos PDFs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>FNP</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Qualidade da base</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Erros de grafia ('AAntônio João' MS, 'CanaBrava do Norte' MT); DF ausente; SP com 590 municípios (de 645). Cruzar por chave normalizada e validar com código IBGE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Próximos passos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>O que falta</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>1) PDFs do Atlas 2023 e 2025 (anexar ou liberar www.gov.br na rede). 2) Conferir Excel x PDF (prioridade MT, 18 linhas VTN&gt;VTI de 2025, MRTs de 2023). 3) Extrair municípios por MRT. 4) Calcular sobreposição MRT x região FNP (% em comum, pureza, Jaccard).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -636,7 +897,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8105,7 +8366,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11212,7 +11473,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11945,7 +12206,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13727,7 +13988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>